<commit_message>
Revise weeks 8-10 LinkedIn strategy and update batch config
- Replace LinkedIn posts 4-5 with carousel and native video formats (weeks 8-10)
- Revise podcasts, blog, and social posts across weeks 7-10
- Update content recipe, quarterly plan, brand config, and batch rule
- Add rules/ directory and update batch summary

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/outputs/drafts/content-batch-2026-04-04/content-batch-summary-20260404.xlsx
+++ b/outputs/drafts/content-batch-2026-04-04/content-batch-summary-20260404.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Blog'!$A$1:$H$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Podcast'!$A$1:$H$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Clips'!$A$1:$H$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'LinkedIn'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'LinkedIn'!$A$1:$H$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Facebook'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -705,7 +705,7 @@
 Consider how most surgeons manage their financial structure. There's a CPA who handles the tax return. There's an advisor (or maybe a 401(k) from a prior employer) managing investments. There might be an attorney who drafted an estate plan a few years ago. Each of these professionals is competent in their domain. And each of them is seeing only one piece of the picture.
 The CPA sees tax compliance. The advisor sees the investment portfolio. The attorney sees the estate documents. But who is looking at how these pieces interact? Who is checking whether the S-Corp salary calibration is optimized against retirement plan capacity? Whether the investment allocation is coordinated with the tax strategy? Whether the estate plan reflects the current entity structure?
 In most cases, nobody. And the gaps between these silos are where the biggest opportunities (and the biggest leaks) tend to live.
-This is what a financial second opinion is designed to catch. Not the things your current advisors are doing wrong, but the things that fall between them.
+This is what a financial second opinion is designed to catch: the things that fall between your advisors, in the gaps where no single professional has a clear line of sight.
 ## What a Financial Second Opinion Actually Covers
 A meaningful second opinion isn't a sales pitch disguised as a review. It's a structured, independent assessment of four interconnected areas that together determine how much of your income you actually keep and how efficiently your wealth compounds.
 ### Area 1: Entity Structure
@@ -720,7 +720,7 @@
 A second opinion looks at effective tax rate benchmarking (what should your rate be at your income level, and how does yours compare?), income timing and character strategies (are you converting income that could be capital gains into ordinary income through structural decisions?), and coordination between your personal and practice-level tax strategies.
 ### Area 4: Investment Allocation
 This isn't about picking better stocks. It's about whether your investment allocation is coordinated with your overall financial structure. Are taxable accounts holding tax-inefficient assets that should be in retirement accounts? Is your portfolio risk level calibrated to your timeline and liquidity needs? Are you harvesting losses systematically, or only when your advisor remembers?
-The coordination between investment strategy and tax strategy is where many advisors leave value on the table, not because they're bad at investing, but because they're not looking at the tax picture simultaneously.
+The coordination between investment strategy and tax strategy is where many advisors leave value on the table. They are strong investors. They are simply working from a portfolio screen, not a tax return, when they make allocation decisions.
 ## The Math: What a Second Opinion Can Reveal
 Let's walk through a scenario to make this concrete.
 Consider a surgeon earning $850,000 through an S-Corp, with a CPA-recommended strategy that includes a 401(k) contribution of $31,000 (the 2026 maximum with catch-up), a SEP contribution, and individual investment accounts managed by a separate financial advisor.
@@ -744,7 +744,7 @@
 ## The Surgical Parallel, One More Time
 You already know why second opinions work. You've been on both sides of them. You've ordered them when the imaging was ambiguous. You've provided them when a colleague wanted a fresh perspective.
 You know that the best surgeons welcome second opinions because they understand the stakes of getting it wrong. And you know that the value isn't in contradicting the first reading. It's in completeness. In catching what the first reader, through no fault of their own, wasn't positioned to see.
-Your financial structure deserves the same discipline. Not because your current advisors are failing you. But because the complexity of surgeon-level financial planning, where entity design, retirement vehicles, tax strategy, and investment allocation all interact, is exactly the kind of case where a second set of eyes reveals findings that no single reader would catch alone.
+Your financial structure deserves the same discipline. The complexity of surgeon-level financial planning, where entity design, retirement vehicles, tax strategy, and investment allocation all interact, is exactly the kind of case where a second set of eyes reveals findings that no single reader would catch alone.
 April 15 arrives this week. Whether you're filing or extending, this is a natural moment to step back and ask a simple question: has anyone ever looked at my full financial picture with the same diagnostic rigor I bring to complex cases?
 If the answer is no, the second opinion is free to request. The findings, as the math shows, tend to pay for themselves many times over.
 Capably Yours,
@@ -1143,7 +1143,7 @@
 Today, I want to give you the calendar.
 ---
 ## INTRO AND CONTEXT (1-2 minutes)
-Here's the reality. The months between April 15 and October 15 are the most valuable planning period of the financial year. Not because there are deadlines breathing down your neck (the opposite, actually). But because this is when you have current-year data, time to implement, and no deadline pressure forcing reactive decisions.
+Here's the reality. The months between April 15 and October 15 are the most valuable planning period of the financial year. The deadlines are behind you. Current-year data is arriving. You have time to implement, and nothing is forcing reactive decisions.
 Tax season, by contrast, is reactive. You're looking backward at a year that already happened, trying to minimize a bill that's already been calculated. April through October is proactive. You're looking forward, building the structure that will determine next year's bill before it ever gets calculated.
 And yet most surgeons treat this period as dead time. Nothing happens between April 15 and the year-end push. That's the gap we're closing today.
 I'm going to walk through four specific financial moves, each with a clear deadline, that are best initiated during this window. These aren't theoretical. They're the same moves that, in practice, separate the surgeons who build wealth efficiently from the ones who feel like they should have more to show for their income. Let's get into it.
@@ -1285,7 +1285,7 @@
 ---
 ## COLD OPEN (30-60 seconds)
 I'm about to say something that might sound self-serving coming from a financial advisor: I think every surgeon should get an independent second opinion on their financial plan.
-Not because your current advisor is bad. Not because your CPA is missing something obvious. But because the cost of not getting one, at your income level, is too high to leave to assumption.
+Your current advisor may be excellent. Your CPA may be catching everything in their lane. The cost of skipping an independent second read, at your income level, is still too high to leave to assumption.
 You already know this intuitively. You've built an entire career around the principle that a second set of eyes catches what the first set misses. Complex imaging, ambiguous pathology, a surgical plan that doesn't sit quite right. You pick up the phone. You send the study. You ask a colleague to take a fresh look.
 You do this because the stakes are high enough to warrant it. Your financial structure carries the same stakes. And yet most surgeons have never subjected it to the same discipline.
 Today, I want to walk through why a financial second opinion matters, what it should cover, what it shouldn't look like, and how to tell the difference between a genuine review and a disguised sales pitch. Let's get into it.
@@ -1293,7 +1293,7 @@
 ## INTRO AND CONTEXT (1-2 minutes)
 April 15 falls this week. Whether you filed, extended, or are wrapping things up right now, this is one of those natural inflection points where it's worth stepping back from the compliance work and asking a broader question.
 That question is simple: has anyone ever looked at my full financial picture, all at once, with fresh eyes?
-For most surgeons, the answer is no. And that's not because they're careless. It's because the way financial services are structured creates silos. Your CPA does your taxes. Your advisor manages your portfolio. Your attorney handles your estate plan. Each one does their job well. But nobody is looking at how those pieces interact.
+For most surgeons, the answer is no. The reason is structural, not personal. Financial services are built in silos. Your CPA does your taxes. Your advisor manages your portfolio. Your attorney handles your estate plan. Each one does their job well. Nobody is looking at how those pieces interact.
 The clinical analogy is exact. Imagine sending a patient's knee MRI to an orthopedist, their bloodwork to an internist, and their cardiac history to a cardiologist, but never having a single physician look at all three together. You'd never practice medicine that way. But most surgeons manage their finances exactly that way.
 The financial second opinion is the integrated read.
 ---
@@ -1350,7 +1350,7 @@
 ## LISTENER TAKEAWAY (1-2 minutes)
 If you take one thing from this episode, let it be this.
 You already practice the discipline of seeking second opinions where the stakes are high. You do it in clinical practice because you know that completeness matters more than confidence. A second perspective catches what the first one, through no fault of its own, wasn't positioned to see.
-Apply that same discipline to your financial structure. Not because your advisors are failing you. But because the complexity of surgeon-level planning, where entity design, retirement vehicles, tax strategy, and investment allocation all interact, is exactly the kind of case where a second set of eyes changes the outcome.
+Apply that same discipline to your financial structure. Surgeon-level planning, where entity design, retirement vehicles, tax strategy, and investment allocation all interact, is exactly the kind of case where a second set of eyes changes the outcome.
 April 15 falls this week. Whether you're filing or extending, this is a natural moment to ask one question: has anyone ever looked at my full financial picture, all at once, with fresh eyes?
 If not, the second opinion is worth requesting. The math tends to make the case on its own.
 ---
@@ -1687,7 +1687,7 @@
 ---
 ## PHILOSOPHICAL CLOSE (1-2 minutes)
 You built your practice with precision, skill, and an enormous investment of your best years. It represents not just financial value, but professional identity, community standing, and the tangible result of decades of training and work.
-It deserves to be treated with the same financial rigor you'd apply to any asset of its size. Not because the practice is "just an investment" (it's far more than that), but because the financial decisions surrounding it affect everything else in your life. Your retirement security. Your family's future. Your ability to choose what comes next on your own terms.
+It deserves to be treated with the same financial rigor you'd apply to any asset of its size. The practice is far more than an investment. And the financial decisions surrounding it affect everything else in your life. Your retirement security. Your family's future. Your ability to choose what comes next on your own terms.
 The question isn't whether you'll exit your practice eventually. You will. Every surgeon does. The question is whether that exit will be on your terms, at a time of your choosing, with a structure that preserves the value you've built. Or whether it will be reactive, compressed, and shaped by circumstances you didn't anticipate.
 Concentration risk is the gap between those two outcomes. Closing that gap starts with seeing it clearly.</t>
         </is>
@@ -2570,7 +2570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>You've Ordered Hundreds of Second Opinions. Have You Gotten One on Your Financial Plan?</t>
+          <t>Week 8 — LinkedIn Carousel Outline (PDF, mechanism post support)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -2933,37 +2933,36 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>LinkedIn Post</t>
+          <t>LinkedIn Carousel Outline</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Opens the week's LinkedIn sequence with the core surgical parallel. The question format creates immediate personal relevance for any surgeon scrolling LinkedIn during tax week. Drives curiosity about what a financial second opinion reveals and positions the blog as the deeper resource.</t>
+          <t>Optional PDF carousel for tactical screening content. Export as portrait slides (1080x1350 or LinkedIn PDF carousel spec). Rule 12 in `rules/linkedin-content-creation-guidelines.md`.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>You've ordered hundreds of second opinions in your career. Have you ever gotten one on your financial plan?
-In clinical practice, the second opinion is standard for complex cases. You send the imaging. You ask a colleague for a fresh read. You do this because the stakes are high enough that a second perspective makes the outcome better.
-Your financial structure carries similar stakes. At surgeon income levels, an independent review of tax strategy, entity structure, retirement plan design, and investment allocation typically identifies $50,000 or more in annual optimization.
-The value of a financial second opinion, just like a clinical one, isn't in contradicting your current advisors. It's in catching what falls between the silos: the interactions between your CPA's tax work, your advisor's portfolio, and your attorney's estate plan that no single professional is positioned to see.
-The same discipline that makes you a better surgeon applies here. Seeking another perspective isn't doubt. It's diligence.
-When was the last time someone looked at your full financial picture with fresh eyes?</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Quote card
-Rationale: The hook question is the post's strongest standalone line. A clean quote card lets the question itself stop the scroll and prompt self-reflection before the reader even engages with the post body.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Charcoal (#1E2428). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "You've ordered hundreds of second opinions in your career." in Playfair Display Medium, approximately 28pt, Off-White (#F6F7F5), centered horizontally, positioned in the upper-center area, maximum width 75% of canvas, line height 1.5. Secondary text: "Have you ever gotten one on your financial plan?" in Playfair Display Medium, approximately 28pt, Antique Gold (#B08D57), centered horizontally, 32px below primary text, maximum width 75% of canvas, line height 1.5. A thin horizontal rule (1px, Blue Slate #5F7483) spans 25% of the canvas width, centered horizontally, 48px below secondary text. Bottom-right corner: Capable Wealth logo mark in Warm Gray (#9AA3A8), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: reflective, provocative, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "You've ordered hundreds of second opinions in your career." in Playfair Display Medium, ~28pt, Off-White (#F6F7F5), upper-center. "Have you ever gotten one on your financial plan?" in Playfair Display Medium, ~28pt, Antique Gold (#B08D57), below. Capable Wealth logo in Warm Gray, bottom-right.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
+          <t>## Slide outline
+1. **Title:** "$225K of capacity reading zero is a silo finding" — sub: "How to tell diagnosis from a pitch"
+2. **The gap:** Three professionals, three lenses; money leaks in the handoffs, not in any single report.
+3. **Red flag 1:** "Move assets before the analysis ends."
+4. **Red flag 2:** "You're not optimized" with no dollar findings.
+5. **Red flag 3:** "Fire your CPA first" before a written memo exists.
+6. **Green flag 1:** Fee for analysis; no custody requirement to hear findings.
+7. **Green flag 2:** Line-item dollars: contributions, brackets, cash flow.
+8. **Green flag 3:** Roadmap your existing team can run together.
+9. **Close:** "Which red flag would show up first in your last review?" (mirrors text post question)
+---
+## Design notes
+- Palette: Capable Wealth only; one Antique Gold accent per slide max.
+- Typography: Playfair for titles, Inter for body; large mobile-readable type.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>week-8-linkedin-1.md</t>
+          <t>week-8-linkedin-carousel.md</t>
         </is>
       </c>
     </row>
@@ -2975,7 +2974,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Your CPA Is Great at Compliance. Your Advisor Is Great at Investments. Who's Looking at the Whole Picture?</t>
+          <t>Week 8 — LinkedIn Native Video (Financial second opinion)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -2985,201 +2984,192 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
+          <t>LinkedIn Native Video</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Native upload for separate LinkedIn distribution lane. Pulls from the week’s podcast/second-opinion theme: silo gap and dollar magnitude. Captions on; no YouTube link in post copy.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>## Production Notes
+- **Format:** 1080x1920 vertical or 1:1 if trimming for feed tests; upload file directly to LinkedIn.
+- **Captions:** Burn in or use LinkedIn auto-captions; first line on screen should match opening hook below.
+- **Cover frame:** Single line on screen: "$50K–$80K often sits between advisors" (Antique Gold on Deep Muted Blue, Capable Wealth type).
+---
+## On-camera script (~60 seconds)
+"$50,000 to $80,000 in Year-one findings often sits between your CPA, your advisor, and your attorney. Each professional did their job. The gap shows up where nobody runs one model that connects tax, retirement, and investments.
+Your CPA sees the return. Your advisor sees the portfolio. Your attorney sees the documents. The expensive part is the handoff.
+A real second opinion ends with dollars on the page and a roadmap your current team can execute. A sales pitch ends with a transfer form.
+If you want one question to run this month: when did someone last read the whole film instead of three separate slices?"</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>week-8-linkedin-native-video.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="120" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Week 8 (April 13–19)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>$50K–$80K Usually Sits Between Your Advisors, Not Inside Them</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>The financial second opinion: are you getting one?</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Second LinkedIn post of the week, extending the second opinion argument from "get one" to "get a coordinated one." Addresses the common objection that the surgeon already has advisors by reframing the problem as a coordination gap, not a competence gap. Publishes mid-week after April 15 has passed.</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Your CPA is great at compliance. Your advisor is great at investments. But who's looking at the whole picture?
-Most surgeons have competent financial professionals. The issue is that those professionals are working in silos. The CPA sees the tax return. The advisor sees the portfolio. The attorney sees the estate documents. Each one optimizes their piece. And the gaps between those pieces are where the biggest opportunities tend to live.
-Here's how this plays out. Consider a surgeon earning $850,000 whose CPA recommends keeping the S-Corp salary at $280,000 to minimize payroll taxes. Smart advice from a tax perspective. But that $280,000 W-2 also caps the cash balance plan contribution formula. The payroll tax savings: about $9,000 per year. The lost retirement plan capacity: potentially $40,000 per year.
-The CPA made a sound call within their domain. The domain was just too narrow.
-A financial second opinion looks at these interactions. Entity structure, retirement plan design, tax strategy, and investment allocation, not as four separate domains, but as a single integrated system.
-The best outcome of that review? Your existing team gets a better roadmap. Nobody gets fired. Everybody gets coordinated.</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Hook post. Opens with silent-loss dollars in the coordination gap between CPA, advisor, and attorney. Positions a coordinated second read as diagnostic, not a personnel swap. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>$50,000 to $80,000 in first-year findings often sits between your CPA's return, your advisor's portfolio, and your attorney's documents. Each professional did their job. The gap exists where nobody owns the full wiring diagram.
+Your CPA optimizes the filing. Your advisor optimizes the allocation. Your attorney optimizes the documents. Each piece can look correct while the handoffs leak: retirement capacity versus salary, loss harvesting versus gain recognition, entity cash flow versus what actually lands on your 1040.
+At surgeon income levels, that coordination gap routinely shows up as six-figure money left on the table in Year 1 alone. Most high earners only see it after a life event forces everyone into one room.
+The return shows one slice. The portfolio statement shows another. The operating agreement shows a third. None of them fail on their own. They fail to meet in one model.
+A coordinated second read is the financial version of a second look at complex imaging. The point is not to replace your team. It is to name where the case was read in slices instead of as one film.
+When was the last time someone reviewed tax, retirement, investments, and entity structure in the same sitting and gave you dollar amounts for what was misaligned?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The dollar range is the scroll-stopper per LinkedIn guidelines. One stat-forward card for Tuesday hook.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text with generous margins (minimum 120px all sides). Primary text: "$50K–$80K" in Playfair Display SemiBold, approximately 88pt, Antique Gold (#B08D57), centered, upper third. Secondary text: "Year 1, often between siloed advisors" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered, 20px below. Thin horizontal rule (1px, Warm Gray #9AA3A8), 30% width, centered, 40px below. Bottom-right: Capable Wealth logo in Off-White, 32px from edges, ~80px wide. Palette only: #243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8. No gradients, no photos.
+Text overlay: As in prompt.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>week-8-linkedin-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Week 8 (April 13–19)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>$9,000 Saved on Payroll. $40,000 a Year Left in Plan Capacity.</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>The financial second opinion: are you getting one?</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Story post. Illustrative S-Corp salary versus retirement capacity trade, framed as coordination miss, not incompetence. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>$9,000 a year saved on payroll tax. About $40,000 a year left unused in retirement plan capacity. The same salary decision can produce both.
+Consider a surgeon earning $850,000 through an S-Corp. The CPA recommends a $280,000 W-2 to trim payroll tax. Reasonable within the lane they were asked to patrol. That salary also feeds formulas that cap how much can ride into a cash balance design.
+Payroll tax savings land on this year's return. The forgone deferral room compounds quietly unless someone models both sides on one page. Five years of that gap is easy math nobody prints on a K-1 summary.
+The CPA was not wrong for the question they were hired to answer. The advisor was not wrong for building the portfolio they were handed. The expensive part is that nobody priced the trade in one place.
+That is the kind of interaction a real second opinion maps. Not who to fire. Where the silos touch.
+Do you know whether your salary was set for payroll tax alone, for plan capacity alone, or for both in the same model?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Conceptual photograph
-Rationale: A photograph of professional documents or folders spread across a desk, each clearly separate, reinforces the "silos" theme visually. The physical separation of materials mirrors the conceptual separation between advisors.
-AI image prompt: Create a 1080x1080px square image. A top-down (bird's eye) view of a clean wooden desk with three distinct stacks of professional documents, each separated by several inches of open desk space. The stacks suggest different professional domains: one with a calculator and financial pages, one with legal-sized documents, one with a portfolio report. No faces, no hands, no people visible. The desk is well-lit with soft, even overhead lighting. Minimal props: a single pen resting between two stacks. Color grading: warm midtones leaning toward Off-White (#F6F7F5), desk surface pulling toward Antique Gold (#B08D57) warmth, document shadows shifted toward Deep Muted Blue (#243A4B). Shallow depth of field with the center stack sharpest and the outer stacks slightly soft. No text, no logos, no graphic overlays. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8) should dominate color grading, 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling. Mood: organized but fragmented, deliberate, thought-provoking. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Rationale: Wednesday story post; desk with separated document stacks reinforces silo theme without literal clinical imagery.
+AI image prompt: Create a 1080x1080px square image. Top-down view of a clean wooden desk with three distinct stacks of professional documents, each separated by open space; one stack with calculator and financial pages, one with legal-sized paper, one with a portfolio summary. No faces, no hands. Soft overhead light; color grading weighted to Off-White (#F6F7F5), Deep Muted Blue (#243A4B) shadows, subtle Antique Gold (#B08D57) warmth. Shallow depth of field. No text or logos on image. Capable Wealth palette only for grading. Photorealistic, not illustrated.
 Text overlay: None
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>week-8-linkedin-2.md</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="120" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Week 8 (April 13–19)</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>The $50K–$80K Finding That Lives Between Your Advisors</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>$225,000 of Capacity Reading Zero Is a Silo Finding, Not an Insult</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>The financial second opinion: are you getting one?</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Third LinkedIn post of the week. Isolates the blog's math example as a standalone insight: the three findings from a second-opinion review that together produce $50K-$80K in Year 1 value. The dollar range is the scroll-stopper; the three findings provide the credibility. Publishes Thursday, post-April 15.</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>A financial second opinion at surgeon income levels typically reveals findings in the $50,000 to $80,000 range. In Year 1.
-Here's how those numbers break down in a common scenario.
-Consider a surgeon earning $850,000 with a 401(k) maxed at $31,000, a SEP contribution, and individual investment accounts managed by a separate advisor.
-Finding 1: Cash balance plan opportunity. No cash balance plan in place. Adding one allows $150,000 to $250,000 in additional tax-deferred contributions per year. At a 42% combined marginal rate, the immediate tax savings on $200,000 in sheltered income is $84,000.
-Finding 2: SEP restructuring. The existing SEP conflicts with the 401(k) employer contribution. Restructuring it into a profit-sharing component frees up $15,000 to $25,000 in additional contribution capacity.
-Finding 3: Tax-loss harvesting coordination. $180,000 in unrealized losses sitting in individual accounts, never harvested because the advisor and CPA don't coordinate. Systematic harvesting saves approximately $43,000 in capital gains taxes.
-None of these findings reflect badly on any individual professional. The CPA wasn't asked about retirement plan design. The advisor wasn't looking at the tax return. The opportunities existed in the spaces between them.
-That's the math on a single, structured review.</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Mechanism post. Practical screen between a diagnostic second opinion and an asset-gathering pitch. Single tactical framework. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>$225,000 of plan capacity showing zero on a coordinated read is a silo finding. It is not proof your CPA failed. It is proof nobody ran one model that connected the pieces.
+A real second opinion ends with numbers tied to line items and tradeoffs. A sales process ends with a transfer form. If the meeting ends with paperwork instead of a written findings memo, you already know which one you got.
+Three pitch signals: they need assets moved before the analysis is finished; the takeaways are mood without math; the first move is to fire someone you already trust.
+Three diagnostic signals: you pay for the work product, not custody; findings read like contribution room, tax brackets, and cash flow; the write-up helps your current team execute together.
+The same screening standard you apply to a new device rep belongs here. Show me the data, show me the mechanism, show me the downside if I say no.
+If you cannot get dollars on the page, you are not getting a second read. You are getting a funnel.
+Which of the three pitch signals would have shown up first in your last "financial review"?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Simple infographic
-Rationale: The three findings are the post's core content. A clean numbered list infographic makes the structure scannable and reinforces the idea that a second opinion produces specific, quantified results, not vague advice.
-AI image prompt: Create a 1080x1080px square social media infographic. Background: Off-White (#F6F7F5). Layout: three rows stacked vertically with equal spacing, each representing one finding. Each row contains a left-aligned number circle (36px diameter, filled Deep Muted Blue #243A4B, number in Off-White #F6F7F5, Inter SemiBold 16pt) and right-aligned text block. Row 1: number "1", heading "Cash Balance Plan" in Inter SemiBold, 16pt, Charcoal (#1E2428), descriptor "$150K–$250K in additional tax-deferred capacity" in Inter Regular, 13pt, Blue Slate (#5F7483). Row 2: number "2", heading "SEP Restructuring" in same style, descriptor "$15K–$25K in freed contribution room" in same style. Row 3: number "3", heading "Tax-Loss Harvesting" in same style, descriptor "$43K in capital gains tax savings" in same style. Top of canvas, centered: "What a Financial Second Opinion Reveals" in Playfair Display Medium, approximately 20pt, Deep Muted Blue (#243A4B). Below the three rows, centered: "Year 1 Value: $50K–$80K" in Playfair Display SemiBold, approximately 22pt, Antique Gold (#B08D57). Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. Generous margins (minimum 80px all sides). No 3D effects, no gradients, no decorative elements. Brand constraints: only Capable Wealth palette, 60/30/10 ratio. Mood: precise, credible, data-driven. Professional financial infographic for orthopedic surgeons ages 45-65.
-Text overlay: As specified in prompt. Headings in Charcoal, descriptors in Blue Slate, value callout in Antique Gold.
+Rationale: Thursday mechanism; red versus green flags as scannable list (palette-true, no neon red; use Deep Muted Blue and Antique Gold accents).
+AI image prompt: Create a 1080x1080px square infographic. Background Off-White (#F6F7F5). Title: "Second opinion or sales pitch?" Playfair Display Medium ~22pt Charcoal (#1E2428), centered. Two columns below: left header "Signals of a pitch" Inter SemiBold 16pt Blue Slate (#5F7483); right header "Signals of a diagnostic" Inter SemiBold 16pt Antique Gold (#B08D57). Three bullet rows each side, Inter Regular 13pt Charcoal, concise phrases: Left: move assets before analysis completes; vague "not optimized" with no dollars; immediate advice to fire your CPA. Right: fee for analysis without custody requirement; findings with line-item dollars; roadmap that coordinates existing professionals. Logo Charcoal, bottom-right, ~60px. Margins 80px. Only Capable Wealth palette.
+Text overlay: As in prompt.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>week-8-linkedin-3.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="120" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Week 8 (April 13–19)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>April 15 Just Passed. Before You Move On, Ask This One Question.</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>The financial second opinion: are you getting one?</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Fourth LinkedIn post of the week. Publishes Thursday or Friday, after April 15. Uses the post-deadline exhale as a natural entry point: before you close the tax chapter and move on, ask whether anyone has ever looked at the full picture. Bridges the second opinion theme to the Week 7 six-month window content by reminding surgeons that the planning window is open.</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>April 15 just passed. You filed or extended. The CPA is going quiet. And there's a natural instinct to close the financial chapter and move on.
-Before you do, one question worth sitting with:
-Has anyone ever looked at your full financial picture, all at once, with fresh eyes?
-Not your tax return in isolation. Not your portfolio in isolation. Not your estate plan in isolation. The whole system: how your entity structure feeds your retirement plan capacity, how your retirement contributions affect your tax rate, how your investment allocation coordinates (or doesn't) with your tax strategy.
-Most surgeons have never had that integrated review. And the gaps in coordination between their CPA, advisor, and attorney are typically where $50,000 to $80,000 in annual value sits uncaptured.
-The window between now and October 15 is the best time of year for that kind of review. No deadlines breathing down your neck. Current-year data coming in. Enough runway to implement changes that actually matter for this tax year.
-One question. One review. It might be the most productive financial conversation you have all year.</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Conceptual photograph
-Rationale: A photograph of a professional in a moment of quiet reflection (looking out a window, seated in a calm office) reinforces the post-deadline pause. The mood should convey thoughtfulness and forward-looking intention, not urgency.
-AI image prompt: Create a 1080x1080px square image. A mid-career professional (male, mid-50s, wearing a clean button-down shirt, no lab coat, no scrubs) seated in a modern office chair, turned slightly toward a large window. He is looking out the window, seen from the side at a three-quarter angle. The window shows soft, diffused natural light with an abstract outdoor scene (trees, sky). The office is minimal: a clean desk behind him, no clutter. No medical equipment, no hospital setting. Calm, reflective posture. Color grading: cool midtones shifted toward Blue Slate (#5F7483), warm highlights from the window light leaning toward Off-White (#F6F7F5) with golden warmth suggesting Antique Gold (#B08D57). Shadows pulled toward Deep Muted Blue (#243A4B). Shallow depth of field with the subject sharp and the background softly blurred. No text, no logos, no overlays. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8) should dominate color grading, 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling. Mood: reflective, calm, forward-looking. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: None
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>week-8-linkedin-4.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="120" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Week 8 (April 13–19)</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>How to Tell a Genuine Financial Review from a Sales Pitch in a Lab Coat</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>The financial second opinion: are you getting one?</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Fifth and final LinkedIn post of the week. Provides a practical screening framework for surgeons who are now curious about a financial second opinion but wary of being sold to. Three red flags and three green flags create a decision tool that positions the reader as an informed consumer. Closes the LinkedIn arc for the week.</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Not every "financial second opinion" is actually a second opinion. Some are sales pitches wearing professional packaging.
-Here's how to tell the difference.
-Three red flags:
-1. They want to move your assets before they've finished the review. If the "second opinion" comes with a pitch to transfer accounts, that's asset gathering, not analysis.
-2. The findings are vague. "You're not optimized" is a fortune cookie, not a finding. A genuine review produces specific numbers: "Your cash balance plan capacity is $225,000 and you're using zero of it."
-3. The first recommendation is to fire someone. If the reviewer's immediate advice is to replace your CPA or advisor, they're positioning themselves as the replacement, not providing an independent assessment.
-Three green flags:
-1. Fee-only, no asset requirement. The reviewer charges for the analysis itself, not for managing your money afterward. The payment is for the work, not the relationship.
-2. Specific, quantified findings. Dollar amounts. Tax savings estimates. Contribution capacity gaps. Math, not opinions.
-3. The goal is to enhance your existing team. The best outcome of a second opinion is that your CPA, advisor, and attorney get a better coordinated roadmap. Nobody gets fired. Everybody gets aligned.
-Apply the same scrutiny to a financial review that you'd apply to a colleague's clinical recommendation. The good ones welcome it.</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Split comparison graphic
-Rationale: A side-by-side "red flag vs. green flag" layout creates immediate visual clarity for the evaluation framework. This is the first image type not yet used this week (posts 1-4 used quote card, conceptual photograph, infographic, and conceptual photograph).
-AI image prompt: Create a 1080x1080px square social media graphic. Background: split vertically into two equal halves. Left half: Deep Muted Blue (#243A4B). Right half: Off-White (#F6F7F5). Top center, spanning both halves: "Second Opinion?" in Playfair Display Medium, approximately 24pt. Left portion of title in Off-White (#F6F7F5), right portion in Charcoal (#1E2428). Left half header: "Red Flags" in Inter SemiBold, 18pt, color #D4735E (a muted warm red, close to the palette's warm tones but readable as cautionary), centered in left half, 80px below title. Three left-aligned text items below, each in Inter Regular, 14pt, Off-White (#F6F7F5), with 24px vertical spacing: "Pitch to move your assets", "Vague 'you're not optimized'", "Recommends firing your CPA". Right half header: "Green Flags" in Inter SemiBold, 18pt, Antique Gold (#B08D57), centered in right half, same vertical position. Three left-aligned text items below, each in Inter Regular, 14pt, Charcoal (#1E2428), same spacing: "Fee-only, no asset requirement", "Specific dollar findings", "Enhances your existing team". Bottom center: Capable Wealth logo mark in Blue Slate (#5F7483), 32px from bottom, approximately 60px wide. Generous margins (80px sides, 60px top/bottom). No 3D effects, no gradients. Brand constraints: primarily Capable Wealth palette with the single cautionary red used only for the "Red Flags" label. Mood: clear, protective, empowering. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: As specified in prompt. Title split across halves, red/green flag headers, three items per side.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>week-8-linkedin-5.md</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3195,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>3.5 Years Too Late</t>
+          <t>Week 9 — LinkedIn Carousel Outline (PDF, diligence questions)</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -3215,259 +3205,245 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
+          <t>LinkedIn Carousel Outline</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>## Slide outline
+1. **Title:** "$400K can ride on goodwill allocation" — sub: "Three questions before you trust the multiple"
+2. **Why it matters:** Headline price vs. tax character; footnotes move wires more than slogans.
+3. **Question 1 — Timeline:** "First talk to close, and what structural work was skipped for speed?"
+4. **Question 2 — Goodwill:** "How is personal goodwill documented today, not promised in a footnote?"
+5. **Question 3 — Earnout:** "Year-three economics if volume, staff, or your hours move."
+6. **How to use this:** Write answers before the next conversation; blanks mean priced ambiguity.
+7. **Close:** "Which question breaks the weakest story you heard last?" (mirror text post)
+---
+## Design notes
+- Same brand system as Week 8 carousel; keep slides 5–7 words per line where possible for mobile.</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>week-9-linkedin-carousel.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Week 9 (April 20–26)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Week 9 — LinkedIn Native Video (Five-year exit timeline)</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>The 5-year exit timeline starts now</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Native Video</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Native upload; dollar-led hook on planning compression; aligns with podcast/conference season angle without calendar-only openers in the hook line.</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>## Production Notes
+- **Format:** Vertical 9:16; captions required.
+- **Cover frame:** "$1.4M gap when you compress the timeline" on brand background.
+---
+## On-camera script (~60 seconds)
+"$1.4 million is the illustrated spread between staging an exit over five years and calling the buyer with eighteen months left. Same practice. Different file.
+The buyer does not pay for your story at dinner. They pay for documentation: goodwill, EBITDA, proof the asset runs without you.
+You already stage complex care. You would not skip workup because someone offered a fast OR date.
+Three questions to write down before the next pitch conversation: real timeline and what got skipped, how personal goodwill is documented today, and what the earnout looks like in year three if your hours change.
+If you cannot answer those on paper, you are not looking at a number yet. You are looking at a headline."</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>week-9-linkedin-native-video.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Week 9 (April 20–26)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>$1,400,000 Is the Cost of Compressing a Five-Year Exit Into Eighteen Months</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>The 5-year exit timeline starts now</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Opens the week's LinkedIn sequence with the core provocation: 18 months is too late for exit planning. The $1.4M value gap and the 5-year timeline create the urgency. Drives traffic to the blog's full protocol.</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Most surgeons start thinking about their practice exit 18 months before they want to leave. That's 3.5 years too late.
-Here's what happens in those missing years. Entity restructuring that would have separated personal goodwill (taxed at 23.8%) from enterprise assets (potentially taxed at 40.8%). Revenue diversification that would have increased the EBITDA multiple. Associate recruitment that would have proven the practice runs without the founder.
-None of that can be done in 18 months.
-Consider a surgeon at 55 with a practice valued at $2.8 million. With a 5-year timeline, entity restructuring, goodwill documentation, revenue diversification, and strategic buyer positioning push the exit value to $4.2 million. Without it, the same surgeon at 60 sells for $2.8 million in a compressed timeline with limited leverage.
-The $1.4 million gap between those two outcomes has nothing to do with the market, the buyer, or the negotiation. It comes down to when the planning started.
-Now that conference season is underway and practice transition is the conversation everywhere, it's worth asking: if you want options in five years, what should you be doing now?
-The answer starts with a valuation baseline and an entity structure review. Year 5 activities. The ones most surgeons never get to because they start in Year 2.</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Hook post. Dollar-led loss of optionality from late planning; conference context appears as background noise, not calendar-only hook. Illustrative valuation path per quarterly plan math. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>$1,400,000 is the illustrated gap between staging an exit over five years and rushing the same practice when the letter of intent shows up in eighteen months. Same clinical asset. Different file.
+Consider a 55-year-old with a practice marked around $2.8 million on a clean year. With five years to document goodwill, normalize earnings, and prove the practice runs without the founder, the same operations often clear closer to $4.2 million in a competitive process. Those figures are illustrative, not a forecast, but they show why the calendar matters. Compress that runway and the buyer names the discount, not you.
+The missing seasons are where entity structure gets set, revenue mix diversifies, and a junior surgeon proves transferability. None of that seasons between tax season and a diligence list. Buyers price the file they see, not the story you tell at a reception.
+Conference chatter makes it easy to confuse interest with readiness. Interest is a dinner invite. Readiness is a diligence binder you could hand over tomorrow.
+When you look at your practice today, what single line item would worry you most if diligence opened next quarter?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Stat highlight card
-Rationale: The "3.5 years too late" framing is the post's anchor provocation. A bold stat card with the $1.4M gap makes the cost of delay impossible to scroll past.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "$1.4M" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper third of the canvas. Secondary text: "The cost of starting your exit plan" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, 24px below primary text. Tertiary text: "3.5 years too late." in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, 8px below secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 30% of the canvas width, centered horizontally, 48px below tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: sobering, authoritative, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "$1.4M" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), upper third center. "The cost of starting your exit plan" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "3.5 years too late." in Inter Regular, ~20pt, Off-White (#F6F7F5), below secondary.
+Rationale: Tuesday hook; $1.4M gap as scroll-stopper.
+AI image prompt: Create a 1080x1080px square social media graphic. Background Deep Muted Blue (#243A4B). Center: "$1.4M" Playfair Display SemiBold ~96pt Antique Gold (#B08D57). Below: "Illustrative cost of starting exit planning too late" Inter Regular ~18pt Off-White (#F6F7F5), centered, max width 80%. Thin rule Warm Gray #9AA3A8, 30% width, 40px below. Logo Off-White bottom-right. Palette only Capable Wealth hexes. No stock photos.
+Text overlay: As in prompt.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>week-9-linkedin-1.md</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="120" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Week 9 (April 20–26)</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Your Practice Exit Is a Treatment Plan</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>$2,800,000 on the Term Sheet Today, or $4,200,000 After Five Years of Staging</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>The 5-year exit timeline starts now</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>Second LinkedIn post of the week, shifting from the provocative $1.4M number to the conceptual reframe: a practice exit should be staged like a surgical treatment plan. Uses the clinical metaphor to make the 5-year timeline feel intuitive rather than daunting. Builds on the blog's year-by-year protocol.</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Your practice exit isn't a single event. It's a sequence.
-Think about how you'd approach a complex surgical case. You wouldn't skip the imaging, walk into the OR, and figure it out in real time. You'd stage the treatment. Diagnostics first. Pre-operative planning. Intervention. Recovery protocol.
-A practice transition follows the same logic.
-Year 5 is the diagnostic: valuation baseline and entity structure review. Year 4 is the pre-treatment: personal goodwill documentation and revenue diversification. Year 3 is the intervention: associate recruitment and systematization to prove the practice operates without you. Year 2 is the approach: buyer identification and earnout framework development. Year 1 is the execution.
-Compressing all of that into 12 to 18 months is the financial equivalent of skipping the treatment plan and going straight to the procedure. You might get an acceptable outcome. But you'll almost certainly leave value on the table, because the steps that create the most value (entity restructuring, goodwill documentation, proving transferability) need time to season.
-Conference season has started. If the conversations around practice transition feel overwhelming, start with the diagnostic. A formal valuation and entity structure review. That's the Year 5 activity, and everything else builds from there.</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Story post. Treatment-plan metaphor with concrete numbers; parallels surgical staging to financial exit staging. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>$2,800,000 on a term sheet next year, or $4,200,000 after five years of documented goodwill, cleaner EBITDA, and proof the asset transfers. The spread is not luck. It is timing and file quality.
+You already stage complex cases. Imaging first, plan before the incision, recovery mapped before discharge.
+A practice exit uses the same rhythm. Year 5 is diagnosis: valuation baseline and entity review. Year 4 is pre-treatment: goodwill evidence and revenue mix. Year 3 proves the machine runs without you. Years 2 and 1 are approach and closure.
+Skip the early years and you still close. You just close with fewer bids, thinner documentation, and less room to say no.
+Collapse that arc into twelve months and you are not negotiating from strength. You are accepting the bid that tolerates the holes. The discount is not a mystery fee. It is the market charging you for missing pages.
+The question is not whether you want to sell Monday. It is whether your film set is complete when someone asks to see it.
+What lives in your file today that counts as Year 5 diagnostic work on paper, not in your head?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Conceptual photograph
-Rationale: The treatment plan metaphor calls for an image that bridges the clinical and strategic worlds. A thoughtful professional reviewing documents or a planning-oriented scene reinforces the deliberate, structured approach to exit planning.
-AI image prompt: Create a 1080x1080px square social media image. A close-up of professional hands reviewing a structured document on a clean, modern desk. The document appears to be a planning document with visible section headers and timeline markers (not readable text, just the visual impression of structure). A fountain pen rests beside the document. The desk is walnut or dark wood. Soft, warm directional light from the left creates gentle shadows. Shallow depth of field with the background completely blurred. No faces, no medical equipment, no screens. Color grading: warm midtones leaning toward Off-White (#F6F7F5), cool shadows shifted toward Deep Muted Blue (#243A4B), subtle golden warmth in the highlights suggesting Antique Gold (#B08D57). No text, no logos, no graphic overlays. Brand constraints: only colors from the Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8) should dominate the color grading, following the 60/30/10 ratio. No cartoons, no clip art, no generic stock photography, no clickbait styling. Mood: deliberate, strategic, composed. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Rationale: Wednesday narrative; hands reviewing a structured planning document, no readable text, calm analytical mood.
+AI image prompt: Create a 1080x1080px square image. Close-up of professional hands reviewing a structured document on a modern desk; section headers visible as shapes only, not readable text; fountain pen beside page; walnut desk; soft left light; shallow depth of field; grading toward Off-White (#F6F7F5), Deep Muted Blue (#243A4B) shadows, Antique Gold (#B08D57) highlight hints. No faces, no logos on image. Photorealistic. Capable Wealth palette in grading only.
 Text overlay: None
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>week-9-linkedin-2.md</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="120" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Week 9 (April 20–26)</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Conference Season Filter</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>$400,000 Can Ride on Goodwill Allocation Alone. Three Questions Cut Through the Deck.</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>The 5-year exit timeline starts now</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Third LinkedIn post, timed for peak conference season. Positions Jared as the advisor who prepares surgeons before they get pitched. The three diagnostic questions (timeline, goodwill, earnout) give surgeons a portable evaluation framework for any conference conversation about practice transition. Bridges the anchor's strategic planning message to immediate real-world application.</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Conference season is here. You'll hear more about practice transitions in the next 30 days than in the last 12 months. Here's what to filter for.
-Not every conversation is created equal. The pitch decks are polished. The multiples sound compelling. The word "partnership" will come up more times than you can count. But three questions will tell you more about any deal than 50 slides ever could.
-**Question 1: What was the timeline from first conversation to close?**
-Clean, well-structured deals typically take 9 to 14 months. If the answer is four months, the surgeon likely didn't have time to optimize entity structure, document personal goodwill, or properly evaluate the earnout. Speed benefits the buyer, not the seller.
-**Question 2: How was personal goodwill handled?**
-Personal goodwill is taxed at long-term capital gains rates (23.8%). Enterprise goodwill allocated to certain asset classes can be taxed at ordinary income rates (up to 40.8%). The allocation between them can mean a $300,000 to $500,000 difference on a $4 million sale. If the acquirer treats this as a footnote, they're not optimizing for your outcome.
-**Question 3: What does the earnout structure look like three years out?**
-A headline multiple of 5x means nothing if 40% of the purchase price is contingent on post-sale performance metrics. Ask what happens if you reduce clinical hours. Ask what happens if a key staff member leaves. The three-year view reveals the real deal.
-Timeline tells you the pace. Goodwill tells you the sophistication. Earnout tells you the risk.
-Save these three questions. You'll need them this month.</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Mechanism post. Portable diligence questions with tax magnitude anchor; avoids "conference season is here" as opening. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>$400,000 of tax economics can swing on how goodwill is allocated on a $4 million practice sale. The deck will celebrate the multiple on page one. The allocation table is where your wire transfer meets the IRS.
+Three questions before you treat a pitch like a done deal.
+What was the real timeline from first conversation to close, and what structural work was skipped to protect that speed?
+How is personal goodwill documented today, not promised in a slide footnote?
+What does the earnout look like in year three if your volume, your staff, or your clinical hours shift?
+Write the answers down. If you cannot, you are not ready to nod at a number.
+Speed usually helps buyers. Vague goodwill language helps buyers. Heavy earnouts push risk back to you. If you cannot get plain answers at the first meeting, assume the ambiguity was priced in before you sat down.
+Treat it like a multidisciplinary case conference. Data first, story second.
+Which of the three questions would have broken the weakest part of the last deal story you heard?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Simple infographic
-Rationale: The three questions are a portable framework. An infographic makes them scannable, saveable, and shareable, which is exactly how this content should function during conference season.
-AI image prompt: Create a 1080x1080px square social media infographic. Background: Off-White (#F6F7F5). Layout: structured vertical stack with generous margins (minimum 80px all sides). Top of canvas: "Conference Season Filter" in Playfair Display Medium, approximately 28pt, Charcoal (#1E2428), centered. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 40% of canvas width, centered, 20px below title. Below accent line: subtitle "3 questions before any deal conversation" in Inter Regular, 14pt, Blue Slate (#5F7483), centered, 16px below accent. Three content blocks stacked vertically, each 160px tall, separated by 20px. Each block has a left-aligned number in Playfair Display SemiBold, 48pt, Antique Gold (#B08D57), with label text in Inter SemiBold, 16pt, Charcoal (#1E2428) to the right of the number, and description text in Inter Regular, 13pt, Blue Slate (#5F7483) below the label. Block 1: "Timeline" / "What was the timeline from first conversation to close?" Block 2: "Goodwill" / "How was personal goodwill handled in the deal?" Block 3: "Earnout" / "What does the earnout look like at Year 3?" Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 32px from edges, approximately 60px wide. No 3D effects, no chart junk, no gradients, no illustrations. Brand constraints: only Capable Wealth palette, 60/30/10 ratio. Mood: structured, practical, authoritative. Professional financial infographic for orthopedic surgeons ages 45-65.
-Text overlay: Title, subtitle, and three numbered question blocks as specified in the prompt.
+Rationale: Thursday mechanism; three-question filter as saveable graphic.
+AI image prompt: Create a 1080x1080px square infographic. Background Off-White (#F6F7F5). Title "Three diligence questions" Playfair Display Medium ~24pt Charcoal (#1E2428), centered. Subtitle "Before you trust the headline multiple" Inter Regular 14pt Blue Slate (#5F7483). Three stacked blocks, each: number in Antique Gold (#B08D57) Playfair SemiBold ~40pt left; label Inter SemiBold 16pt Charcoal; line Inter Regular 13pt Blue Slate. (1) Timeline: "First conversation to close, and what got skipped to speed it?" (2) Goodwill: "How is personal goodwill documented, not just described?" (3) Earnout: "Year-three economics if volume, staff, or your hours move?" Logo Charcoal bottom-right. Margins 80px. No chart junk. Capable Wealth palette only.
+Text overlay: As in prompt.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>week-9-linkedin-3.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="120" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Week 9 (April 20–26)</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Personal Goodwill Starts in Year 5</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>The 5-year exit timeline starts now</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Fourth LinkedIn post, isolating the personal goodwill documentation angle from the blog's 5-year protocol. Positions personal goodwill as a Year 4-5 activity that most surgeons discover too late. The $300K-$500K tax savings number creates urgency without fear-mongering. Builds toward the May content arc on personal goodwill (Week 11).</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Your reputation, your referral relationships, your surgical skill. They all have a dollar value. And if you don't document that value before you sell your practice, the IRS will tax it as if it doesn't exist.
-Personal goodwill is the portion of your practice's value that's attributable to you, the individual surgeon, rather than to the business itself. It's your reputation, your patient loyalty, your referral network. The value that walks out the door when you do.
-Here's why it matters at the point of sale. Personal goodwill is taxed at long-term capital gains rates: 20% federal plus 3.8% NIIT, for a combined 23.8%. Enterprise goodwill allocated to certain asset classes can be taxed at ordinary income rates: up to 37% federal plus 3.8%, for a combined 40.8%.
-On a $4 million practice sale, the allocation between personal and enterprise goodwill can shift the tax bill by $300,000 to $500,000, based on current tax law.
-But there's a catch. Personal goodwill must be established and documented before the sale process begins. Non-compete agreements, referral source analysis, patient retention data, evidence that the practice's revenue depends on your individual presence. The IRS scrutinizes after-the-fact goodwill claims. Documentation that appears during negotiations, rather than years before them, is far more likely to be challenged.
-This is a Year 4 or Year 5 activity. If you're within five years of a potential practice transition, the documentation process should be underway.
-The surgeons who capture this value aren't doing anything exotic. They're just starting early enough to do it right.</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Conceptual photograph
-Rationale: A different subject from Post 2. An image of a professional document or legal setting (not people) reinforces the documentation theme and the formal, structural nature of personal goodwill preparation.
-AI image prompt: Create a 1080x1080px square social media image. A top-down view of a clean, dark leather-bound portfolio folder open on a walnut desk. Inside the folder, a single sheet of cream-colored paper with the impression of formal text (not readable, just the visual texture of a professional document). A brass pen clip catches warm light. A small stack of additional papers sits beside the folder, slightly offset. The desk surface is visible around the edges with clean negative space. No hands, no faces, no screens. Color grading: deep warm tones with the leather and wood in Charcoal (#1E2428) and Deep Muted Blue (#243A4B), the paper in Off-White (#F6F7F5), the brass detail in Antique Gold (#B08D57). Soft, even lighting from above with minimal shadows. No text, no logos, no graphic overlays. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling. Mood: formal, deliberate, substantial. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: None
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>week-9-linkedin-4.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="120" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Week 9 (April 20–26)</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Options Later Means Leverage Now</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>The 5-year exit timeline starts now</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Closes the week's LinkedIn arc with the philosophical message: starting the planning process creates leverage, not commitment. Addresses the common objection that "thinking about exit planning means I'm ready to leave." Reframes early planning as an act of professional empowerment. Ties back to the podcast's closing message.</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Starting a 5-year exit planning process does not mean you're selling. It does not mean you're committed to a PE deal. And it does not mean you're leaving medicine.
-What it means is that you're building leverage.
-A surgeon who has completed a valuation baseline, documented personal goodwill, diversified revenue, and recruited an associate can evaluate any offer from a position of strength. They can say no. They can wait. They can sell to a hospital system instead of PE. They can bring in a partner and keep operating for another decade. They can retire on terms they designed themselves.
-A surgeon who hasn't done any of that takes whatever's available when they're ready to leave. And "whatever's available" is always worth less than what a prepared seller can command.
-Conference season will bring plenty of conversations about practice transition. Some of them will be worth pursuing. Most of them will be worth filing away. All of them will be more valuable if you've done the foundational work first.
-The best time to start planning your exit is when you have no urgency to leave. That's when every decision is made from strength rather than necessity.
-If that window is open for you right now, use it.</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Quote card
-Rationale: The "options later means leverage now" message is the week's philosophical capstone. A quote card with this framing creates a shareable, memorable close to the LinkedIn arc. This type hasn't been used yet in this week's LinkedIn posts.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Charcoal (#1E2428). Layout: centered text composition with generous margins (minimum 100px all sides). Primary text: "The surgeon who planned ahead always has choices. The surgeon who waited has an offer." in Playfair Display Medium, approximately 30pt, Off-White (#F6F7F5), centered horizontally and vertically, maximum width 75% of canvas, line height 1.5. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 25% of canvas width, centered, 40px below primary text. Attribution text: "Capable Wealth" in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered, 20px below accent line. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: reflective, authoritative, grounding. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: Quote text in Playfair Display Medium, ~30pt, Off-White (#F6F7F5), centered. Attribution in Inter Regular, ~16pt, Warm Gray (#9AA3A8), centered below accent line.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>week-9-linkedin-5.md</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>WEEK 10 (APRIL 27 - MAY 3)</t>
+          <t>WEEK 10 (APRIL 27 – MAY 3)</t>
         </is>
       </c>
       <c r="B23" s="3" t="n"/>
@@ -3481,12 +3457,12 @@
     <row r="24" ht="120" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Week 10 (April 27 - May 3)</t>
+          <t>Week 10 (April 27 – May 3)</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>The PE Pitch Deck Is Missing Four Things</t>
+          <t>Week 10 — LinkedIn Native Video (PE deck / concentration)</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -3496,261 +3472,195 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
+          <t>LinkedIn Native Video</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Optional native clip extending PE and diligence themes for the same week as `week-10-linkedin-1.md` through `week-10-linkedin-3.md`.</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>## Production Notes
+- **Cover frame:** "$1.4M rollover on a $4M headline" — brand colors, high contrast.
+---
+## On-camera script (~60 seconds)
+"$1.4 million of a four-million-dollar headline often sits in rollover equity, not in cash you control this decade. Thirty-five percent rollover is the arithmetic. The deck still leads with the multiple.
+Before you lean in, pull the cap table on that rollover, the comp schedule past year one, and the EBITDA bridge under the multiple. If those stay in the appendix, you are still on marketing, not diligence.
+Separate issue: more than half your net worth in one illiquid line item would force a risk talk in any other portfolio. Your practice deserves the same measurement.
+Two jobs this month: translate the deck into cash, calendar, and control, and write down your practice as a percent of household net worth using a real valuation, not a guess."</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>week-10-linkedin-native-video.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Week 10 (April 27 – May 3)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>$1,400,000 of a $4,000,000 Offer Can Sit Outside Your Cash Control for Years</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Concentration risk: your practice is your biggest bet</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>Opens the week's LinkedIn sequence with the PE pitch deck provocation. Conference season is the perfect backdrop. The "missing four things" structure creates a curiosity gap that drives reads and shares. Drives traffic to the blog for the full analysis.</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Consider a surgeon looking at a PE pitch deck. It's beautiful. The projections are compelling. The word "partnership" is on every page.
-It's also missing four things.
-1. Rollover equity terms. Most deals require 30-35% of the sale price to be reinvested in the acquiring entity. On a $4M deal, that's $1.4M that stays illiquid, in someone else's control, for 3-5 more years.
-2. Compensation adjustments. Post-acquisition, surgeon pay often declines 15-25% through productivity thresholds, management fees, and staffing changes. The Year 1 guarantee is not the long-term reality.
-3. EBITDA normalization. How the buyer calculates your practice's earnings affects both valuation and earn-out targets. If the normalized number is inflated, you're starting behind.
-4. Hold period dynamics. For 3-5 years post-close, you're an employee with new reporting structures, new compensation formulas, and reduced autonomy.
-None of this means the deal is bad. Some PE transactions create genuine wealth and genuine professional opportunity.
-But a pitch deck that emphasizes multiples and "partnership" while de-emphasizing these four elements is incomplete. And conference season is exactly the time to know what's not on the slides before you sit down for dinner.</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Hook post. Rollover equity as illiquid, buyer-favorable structure; challenges deck emphasis versus footnotes. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>$1,400,000 of a $4,000,000 headline often sits in rollover equity, not in your bank account. At 35% rollover, that is the math. Illiquid, timing you do not control, economics set by someone else's next chapter.
+The deck leads with the multiple. It whispers rollover mechanics, post-close compensation resets, how EBITDA was normalized, and what five years inside the platform actually looks like on your W-2.
+Ask for the cap table on the rollover, the pro forma comp schedule past year one, and the actual EBITDA worksheet. Polished slides survive when specifics stay in the appendix. Your job is to promote the appendix to page one.
+None of that makes every transaction wrong. Some partnerships are excellent. It means the headline is not the return. Your job in diligence is to translate the deck into cash, calendar, and control, not into adjectives.
+Before you lean in, write four lines on a notecard: rollover percent and terms, how pay changes after year one, the EBITDA bridge they used, and the hold-period exit options. If two are blank, you are still on page one.
+Which of the four would change your answer if it moved ten percent against you?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Stat highlight card
-Rationale: The "4 things missing" creates a bold, scrollable hook. A clean stat card with the number and context is immediately readable and shareable for the conference-season audience.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "4" in Playfair Display SemiBold, approximately 140pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper third of the canvas. Secondary text: "things missing from" in Inter Regular, approximately 22pt, Off-White (#F6F7F5), centered horizontally, 16px below primary text. Tertiary text: "that PE pitch deck." in Inter Regular, approximately 22pt, Off-White (#F6F7F5), centered horizontally, 8px below secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 30% of the canvas width, centered horizontally, 48px below tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: knowing, precise, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "4" in Playfair Display SemiBold, ~140pt, Antique Gold (#B08D57), upper third center. "things missing from" in Inter Regular, ~22pt, Off-White (#F6F7F5), below primary. "that PE pitch deck." in Inter Regular, ~22pt, Off-White (#F6F7F5), below secondary.
+Rationale: Tuesday hook; 35% of $4M as $1.4M rollover called out as the scroll-stop.
+AI image prompt: Create a 1080x1080px square social media graphic. Background Deep Muted Blue (#243A4B). Primary: "$1.4M" Antique Gold (#B08D57) Playfair SemiBold ~96pt centered upper third. Secondary: "Typical rollover slice on a $4M headline" Inter Regular ~18pt Off-White (#F6F7F5) centered below. Thin Warm Gray rule, 30% width, 40px below. Logo Off-White bottom-right ~80px. Capable Wealth palette only. No photos.
+Text overlay: As in prompt.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>week-10-linkedin-1.md</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="120" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Week 10 (April 27 - May 3)</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Three Numbers Your Practice Appraiser Won't Emphasize</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
+    <row r="26" ht="120" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Week 10 (April 27 – May 3)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>55% of Your Net Worth in One Illiquid Line Item Is a Portfolio Problem Dressed as a Career</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Concentration risk: your practice is your biggest bet</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Conference season sparks valuation conversations. This post positions three under-discussed valuation variables (personal goodwill split, normalized EBITDA, working capital adjustment) as the numbers that actually determine wealth outcomes in a practice sale. Extends the blog's "what they don't tell you" theme into the valuation process itself.</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Valuation day is coming. Whether it's a PE firm's offer, a formal appraisal, or a back-of-the-napkin estimate from a colleague, you'll hear a number. And that number will feel like the answer.
-Here are three numbers your practice appraiser won't emphasize, but your wealth depends on.
-**1. The personal goodwill split.**
-When your practice is valued, the total value gets allocated between enterprise goodwill (the practice's systems, brand, and transferable operations) and personal goodwill (your reputation, referral relationships, and surgical skill). This split determines tax treatment. Enterprise goodwill on certain asset allocations may be taxed at ordinary income rates (up to 40.8%). Personal goodwill can qualify for capital gains treatment (23.8%). On a $4M sale, the difference in tax treatment is $678,000. Your appraiser may not split this at all unless you ask.
-**2. Normalized EBITDA.**
-Buyers don't value your practice based on what your accountant reports as net income. They use normalized EBITDA, which strips out owner-specific expenses (above-market salary, personal vehicles, family members on payroll). This normalized number could be significantly higher or lower than what you expect. And the multiple gets applied to the normalized figure, not the reported one.
-**3. The working capital adjustment.**
-In most practice sales, the buyer expects a certain level of working capital (cash, receivables, supplies) to remain in the business at closing. This is cash you might assume you're keeping but aren't. The working capital target is negotiable, but only if you know it's on the table.
-Conference season is when valuation conversations start. Knowing these three numbers before the conversation gives you leverage in it.</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Story post. Balance-sheet concentration with concrete illustrative weights; practice as largest bet. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>55% of net worth in a single illiquid asset would trigger an immediate risk conversation in any diversified book. Your practice often clears that bar once you mark it honestly.
+Consider a practice at $3 million, home equity at $500,000, investments at $2 million. Total net worth lands near $5.5 million. The practice is the overweight sleeve. It cannot be trimmed monthly. It cannot be rebalanced like an ETF. It pays you well and pins your wealth to one engine. Stress-test the same balance sheet as if the practice value moved down twenty percent and see what is left for everything else you care about funding.
+That is not an insult to what you built. It is the same math you would apply to a stock position of the same size. Familiarity does not reduce variance. Income today does not hedge a binary liquidity event tomorrow.
+The goal is not to force a sale next quarter. The goal is to know the concentration is chosen, measured, and paired with a timeline that preserves optionality.
+What percentage of your household net worth is the practice if you plug in a real valuation, not a mental round number?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Conceptual photograph
-Rationale: A professional appraiser or financial advisor environment conveys the seriousness of valuation without being generic. An image of a clean, modern professional office with financial documents or a laptop on a desk suggests the analytical work behind a valuation.
-AI image prompt: Create a 1080x1080px square image. A clean, modern professional office desk photographed from a slightly elevated angle. On the desk: an open laptop displaying a spreadsheet (content blurred for privacy), a few printed pages of financial reports, a high-quality pen, and a ceramic coffee cup. The desk surface is clean light wood or white laminate. Natural light enters from a large window to the left, casting soft shadows. The background shows a minimal, professional office environment with blurred bookshelves and a potted plant. No people visible. Color grading: cool midtones shifted toward Blue Slate (#5F7483), highlights restrained to Off-White (#F6F7F5) with warm accents from the light suggesting Antique Gold (#B08D57). Shadows pulled toward Deep Muted Blue (#243A4B). Shallow depth of field with the laptop and documents in focus, background blurred. No text, no logos, no graphic overlays. Brand constraints: only Capable Wealth palette colors dominate the grading, 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling. Mood: analytical, precise, professional. Financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Rationale: Wednesday story; analytical desk scene suggesting review of personal balance sheet (blurred spreadsheet).
+AI image prompt: Create a 1080x1080px square image. Slightly elevated angle on light wood desk: laptop with blurred spreadsheet, printed financial pages, quality pen, ceramic mug. Natural window light from left; Blue Slate (#5F7483) cool tones, Off-White (#F6F7F5) highlights, Deep Muted Blue (#243A4B) shadows. No people; no readable text; no logos on image. Photorealistic; Capable Wealth palette in grading.
 Text overlay: None
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>week-10-linkedin-2.md</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="120" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Week 10 (April 27 - May 3)</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>46% of Your Net Worth in One Asset</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
+    <row r="27" ht="120" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Week 10 (April 27 – May 3)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>$678,000 Can Live in Three Lines Your Appraiser Never Highlighted</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Concentration risk: your practice is your biggest bet</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>LinkedIn Post</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Bridges from the PE-specific content in LinkedIn posts 1 and 2 to the broader concentration risk theme. The "you'd never put 46% in a single stock" comparison makes the abstract concept of concentration risk instantly tangible. Positions practice diversification as a strategic priority regardless of PE interest.</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>Your practice is 46% of your net worth. You'd never put 46% of your portfolio in a single stock. So why is your biggest asset the one you've never diversified?
-Here's the math. Consider a surgeon with a practice worth $3M, a home with $500K in equity, and a $2M investment portfolio. Total net worth: $5.5M. The practice represents $3M of that. That's 55%. Even with more generous calculations, you're looking at 46%.
-In any investment portfolio, that level of concentration would trigger immediate action. Rebalance. Diversify. Hedge. No advisor would let a single position dominate half your wealth, especially one that's illiquid, can't be sold in pieces, and depends entirely on one person's ability to work.
-But most practice-owning surgeons have never framed it this way. The practice feels different because it generates income. It feels safe because it's familiar. And it feels permanent because you built it.
-None of those feelings change the underlying portfolio math.
-Three moves reduce concentration risk without requiring a sale:
-Diversify revenue sources within the practice (associates, ASC stakes, ancillary income). Document personal goodwill now (this is worth $678K in tax savings on a $4M sale, and must be done years in advance). Build a transition timeline, even if you're ten years from exiting.
-The goal isn't to rush toward an exit. The goal is to ensure your biggest asset gets the same analytical rigor you'd apply to any investment of its size.</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Mechanism post. Three valuation lines that move tax and cash: goodwill split, normalized EBITDA bridge, working capital target. Execution follows `rules/linkedin-content-creation-guidelines.md`.</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>$678,000 is the illustrated tax spread on some $4 million practice sales when personal goodwill is documented versus when the IRS reads the check as ordinary income. Same headline price. Different footnotes.
+Three lines decide more than the multiple on the cover page.
+Goodwill allocation between personal and enterprise character drives rate, not just bragging rights on the term sheet.
+The EBITDA bridge shows what earnings the multiple actually multiplied, not what your P&amp;L felt like at tax time.
+The working capital target is often cash you assumed you would walk away with but leave in the clinic on the way out.
+If your advisor has never walked you through all three on a whiteboard, you have not finished reading your own sale. That is a scope issue, not an intelligence issue.
+Bank appraisals optimize for credit risk. Your wealth outcome optimizes for allocation, normalization, and closing mechanics. Ask for the tables, not the adjectives. If the answer is a handshake, you do not yet have an answer.
+If diligence opened Monday, which of the three lines is still a blank in your own file?
+#orthopedicsurgeon #orthopedicsurgery #physicianfinance</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Simple infographic
-Rationale: A portfolio allocation visual showing the 46% concentration makes the imbalance immediately visible. A simple pie or bar chart comparing "your practice" to "everything else" creates the visual impact that reinforces the post's argument.
-AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (minimum 100px all sides). Center of canvas: a simple donut chart (outer radius approximately 200px, inner radius 100px). The chart has two segments: a large segment representing 46%, filled with Antique Gold (#B08D57), and the remaining 54%, filled with Blue Slate (#5F7483). Inside the donut center: "46%" in Playfair Display SemiBold, approximately 48pt, Charcoal (#1E2428). Below the chart, two legend items stacked vertically, centered: a small square (12px) of Antique Gold (#B08D57) followed by "Practice" in Inter Regular, 14pt, Charcoal (#1E2428). A small square of Blue Slate (#5F7483) followed by "Everything Else" in Inter Regular, 14pt, Charcoal (#1E2428). Above the chart, centered: "Your Net Worth" in Playfair Display Medium, approximately 22pt, Charcoal (#1E2428). Below: "One illiquid asset." in Inter Regular, 14pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No 3D effects, no chart junk, no decorative elements, no gradients. Brand constraints: only Capable Wealth palette, 60/30/10 ratio. Mood: clarifying, precise, thought-provoking. Professional financial infographic for orthopedic surgeons ages 45-65.
-Text overlay: "Your Net Worth" in Playfair Display Medium, ~22pt, above chart. "46%" inside donut in Playfair Display SemiBold, ~48pt. Legend labels and "One illiquid asset." subtext as specified.
+Rationale: Thursday mechanism; three-line diligence checklist.
+AI image prompt: Create a 1080x1080px square infographic. Off-White (#F6F7F5) background. Title "$678K can hide in three lines" Playfair Medium ~22pt Charcoal (#1E2428) centered. Small caption line below title in Inter Regular 11pt Blue Slate: "Illustrative tax spread example, not a promise of results." Three rows: (1) Personal vs enterprise goodwill allocation and tax character. (2) Normalized EBITDA bridge the multiple actually hits. (3) Working capital target and cash left in the business at close. Each row: number circle Deep Muted Blue (#243A4B) with Off-White numeral, text Inter Regular 14pt Charcoal, subline Blue Slate (#5F7483). Logo Charcoal bottom-right. Margins 80px. Capable Wealth palette only.
+Text overlay: As in prompt.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>week-10-linkedin-3.md</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="120" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Week 10 (April 27 - May 3)</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>$678,000 on a Single Planning Decision</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Concentration risk: your practice is your biggest bet</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Isolates the personal goodwill tax math from the blog as a standalone LinkedIn insight. The $678K figure is the week's most shareable number. The post reinforces the critical timing element: documentation must happen years before a sale, which makes this actionable for any surgeon 3-5 years from a potential transition.</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>A $4M practice sale. Two possible tax outcomes. $678,000 apart.
-The only variable: one piece of documentation that most surgeons haven't started.
-Here's the math. Without personal goodwill documentation, the sale proceeds may be taxed at ordinary income rates. At 37% federal plus 3.8% Net Investment Income Tax, that's 40.8%. Tax bill: approximately $1.63M.
-With personal goodwill properly documented before the sale, the proceeds can qualify for long-term capital gains treatment. At 20% federal plus 3.8% NIIT, the rate drops to 23.8%. Tax bill: approximately $952K.
-The difference is $678,000. Same deal. Same price. Same practice.
-Personal goodwill is the value attributable to your reputation, referral relationships, and surgical skill, as distinct from the practice's enterprise value in its systems and equipment. When properly documented, it receives capital gains treatment. When undocumented, the IRS may treat the entire sale as ordinary income.
-The critical timing element: this documentation (non-compete agreements, referral source analysis, patient relationship evidence) must be established years before any transaction. After-the-fact claims get scrutinized and frequently denied.
-If you're within five years of a potential practice transition, of any kind, the personal goodwill conversation should be happening now. The cost of establishing the documentation is minimal. The cost of not having it is $678,000.</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Conceptual photograph
-Rationale: A different visual register from LinkedIn 2's office desk. An image of a surgeon in a reflective moment, perhaps in a conference hallway or looking out a large window, connects the financial planning concept to the human experience of weighing a major life decision.
-AI image prompt: Create a 1080x1080px square image. A professional man (mid-50s, salt-and-pepper hair, wearing a blazer over a button-down shirt, no tie) standing in a modern conference center hallway, looking out through a large floor-to-ceiling window. He is photographed from the side at a slight distance, creating a contemplative mood. Natural daylight enters through the window, casting soft light across his face and the polished floor. The hallway has clean lines, minimal architecture, light-colored walls. No other people visible. He holds nothing in his hands. His expression is thoughtful, not worried. Color grading: cool midtones shifted toward Blue Slate (#5F7483), warm highlights leaning toward Off-White (#F6F7F5) with golden warmth from the window light suggesting Antique Gold (#B08D57). Shadows pulled toward Deep Muted Blue (#243A4B). Shallow depth of field with the man in focus and the far end of the hallway blurred. No text, no logos, no graphic overlays. Brand constraints: only Capable Wealth palette colors dominate the grading, 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait. Mood: contemplative, decisive, professional. Financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: None
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>week-10-linkedin-4.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="120" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Week 10 (April 27 - May 3)</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>What Return Are You Earning on Your Practice?</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>Concentration risk: your practice is your biggest bet</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Closes the week's LinkedIn sequence by reframing practice ownership as an investment that deserves return-on-capital analysis. Shifts the conversation from PE deals and tax strategies to the foundational question: is the return you're earning on this asset commensurate with the risk and concentration? A novel angle most surgeons have never considered.</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>You'd never hold a $3M stock position without knowing your annual return. So what's the return on your practice?
-Here's a question almost no surgeon has been asked. If you treat your practice ownership as an investment of both capital and time, what is the actual return on that investment?
-Let's walk through it. Your practice has a market value (say $3M based on a conservative appraisal). You invest roughly 2,400 clinical hours per year. If your effective hourly take-home is $225, your total annual take-home from the practice is approximately $540K.
-That $540K is the "dividend" your practice pays you. On a $3M asset, that's an 18% annual return. Sounds excellent.
-But now consider the risk profile. This return comes from a single, illiquid, non-diversified asset that depends entirely on your continued health, stable reimbursement rates, local market conditions, and your willingness to show up in the OR every week.
-An 18% return with that risk profile is acceptable. But a diversified portfolio earning 8% with dramatically lower risk, full liquidity, and no dependence on your physical presence produces comparable risk-adjusted returns over a 20-year horizon.
-The point of this exercise isn't to convince you to sell. The point is to analyze. Your practice is likely your biggest asset. It deserves the same financial rigor you'd apply to any investment of comparable size.
-Calculate the return. Assess the risk. And ask yourself whether the concentration is intentional or just something that happened over time.</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Text-based educational card
-Rationale: A clean calculation walkthrough on a card format presents the practice-as-investment math in a scannable, bookmark-worthy format. Different from the stat card in Post 1 and the infographic in Post 3. This is a "save this" style post.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: Off-White (#F6F7F5). Layout: left-aligned text composition with generous margins (100px left, 80px right, 80px top and bottom). Title: "Your Practice as an Investment" in Playfair Display Medium, approximately 24pt, Charcoal (#1E2428), left-aligned, top of content area. Below title, a thin horizontal rule (1px, Antique Gold #B08D57) spanning 40% of canvas width, left-aligned. Below the rule, four rows of calculation text, each row containing a label and value, stacked with 24px spacing: Row 1: "Practice Value:" in Inter Regular, 16pt, Blue Slate (#5F7483), followed by "$3M" in Inter SemiBold, 16pt, Charcoal (#1E2428). Row 2: "Annual Take-Home:" in Inter Regular, 16pt, Blue Slate, followed by "$540K" in Inter SemiBold, 16pt, Charcoal. Row 3: "Implied Return:" in Inter Regular, 16pt, Blue Slate, followed by "18%" in Inter SemiBold, 16pt, Charcoal. Row 4: "Risk Level:" in Inter Regular, 16pt, Blue Slate, followed by "Concentrated, Illiquid, Single-Asset" in Inter SemiBold, 14pt, Antique Gold (#B08D57). Below the four rows, 32px spacing, then: "Is the return worth the risk?" in Inter Medium Italic, 18pt, Charcoal (#1E2428). Bottom-right: Capable Wealth logo mark in Charcoal, 24px from edges, approximately 60px wide. No imagery, no gradients, no 3D effects. Brand constraints: only Capable Wealth palette, 60/30/10 ratio. Mood: analytical, thought-provoking, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: Title, calculation rows, and closing question as specified in the prompt.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>week-10-linkedin-5.md</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H28"/>
+  <autoFilter ref="A1:H27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4188,7 +4098,7 @@
 Second: the existing SEP contribution is conflicting with the 401(k) employer match formula, costing $15,000 to $25,000 in usable contribution room. A simple restructuring eliminates the conflict.
 Third: $180,000 in investment losses have been sitting in taxable accounts for years, unharvested, because the investment advisor and the CPA never compare notes. Systematic harvesting saves roughly $43,000 in capital gains taxes.
 Total value of someone looking at the full picture: $50,000 to $80,000 in Year 1.
-The hard part? Nobody had ever looked. Not because anyone was doing a bad job. But because nobody was doing the same job: seeing how all the pieces connect.</t>
+The hard part? Nobody had ever looked. Every advisor was doing good work in their lane. The gap existed where nobody was doing the same job: seeing how all the pieces connect.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -4342,10 +4252,10 @@
       <c r="F14" s="6" t="inlineStr">
         <is>
           <t>A thought to close out the week.
-The best surgeons welcome second opinions. Not because they doubt their skills. Because they understand that the stakes are high enough, and the cases are complex enough, that completeness matters more than confidence. A second perspective doesn't replace their judgment. It strengthens it.
+The best surgeons welcome second opinions. The stakes are high enough, and the cases complex enough, that completeness matters more than confidence. A second perspective strengthens judgment. It never replaces it.
 The same principle applies to your financial plan.
 If your strategy is sound, a second opinion confirms it. You walk away with the confidence that your structure is working the way it should. If there are coordination gaps between your CPA, your advisor, and your estate plan (and at surgeon income levels, there almost always are), you'd rather know now than discover them years from now, when the compounded cost is much harder to recover.
-Financial planning, at its core, is about the quality of your life. The control you have over your time, your choices, and your future. A plan that's been independently reviewed gives you more of all three. Not because the plan changes dramatically. But because you know, with certainty, that the foundation is solid.
+Financial planning, at its core, is about the quality of your life. The control you have over your time, your choices, and your future. A plan that's been independently reviewed gives you more of all three. The plan may not change dramatically. What changes is your certainty that the foundation is solid.
 The best plans welcome a second look. The best planners do, too.</t>
         </is>
       </c>
@@ -4575,7 +4485,7 @@
 Surgeon B starts planning at 58. Same practice, same market. But with only two years, there's no time to recruit an associate, no time for entity restructuring to season, and no runway to document personal goodwill credibly. At 60, they sell for $2.8 million to the one buyer who's interested, on that buyer's terms.
 Same starting point. Same age at exit. Same market conditions. The difference: $1.4 million.
 That $1.4 million gap has nothing to do with intelligence, surgical skill, or luck. The only variable is when the planning started.
-If you're anywhere in the five-year window, this is the most valuable time you have. Not because you need to make any decisions now, but because the decisions you'll want to make later require groundwork that starts today.</t>
+If you're anywhere in the five-year window, this is the most valuable time you have. The decisions you'll want to make later require groundwork that starts today.</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">

</xml_diff>